<commit_message>
comms: verify the portrait placement question, add PROBE NOTES to the workbook
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Table Smoke Testing.xlsx
+++ b/tasks/The Table Smoke Testing.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROBE NOTES" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +37,17 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -60,13 +72,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,4 +519,64 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:B10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>PROBE NOTES - for lanes, not for Xero</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Traps that have already produced a false test result. Read before writing an automated probe against a generator. Nothing here needs Xero to do anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>1. Anything a probe injects into the page needs class="no-print"</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>A results div appended to document.body is not covered by these generators' print CSS, so it prints as a phantom second page and reads as a layout bug that is not there. This bit the Planet of the Apes sheet, then nearly caused a false report on Walking Dead. Added 2026-09-11 by Character Generators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2. Print output IS reachable headless - print-to-PDF is not a substitute, it is the real thing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Print-to-PDF renders exactly what the print path produces; rasterise it and read it. Only the interactive print dialog and a real printer driver are out of reach. Do not file "needs a real print preview" as a blocker, and do not spend one of Xero's test slots on a paper check that a lane can do itself. Correction recorded 2026-09-11 by Character Generators, after the walkingdead print item was closed this way.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
comms: write the Mothership VTT auth test worksheet, file the three Xero items
Verified the VTT is reachable and the auth form renders before asking him to
test past it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Table Smoke Testing.xlsx
+++ b/tasks/The Table Smoke Testing.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROBE NOTES" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mothership VTT auth 2026-09-12" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,16 +52,29 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -68,11 +82,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +114,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,9 +539,9 @@
       </c>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>No test tabs yet. Comms adds one the moment a lane has something genuinely reachable to verify. If this file has only this sheet, there is nothing waiting on you here.</t>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>One test tab is waiting on you: "Mothership VTT auth 2026-09-12" - the authenticated path on the Mothership VTT. It needs a real account, so only you can run it. Comms verified the site is up and the sign-in form renders before asking. Ten steps, each with what you should see.</t>
         </is>
       </c>
     </row>
@@ -579,4 +622,284 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>MOTHERSHIP VTT - THE AUTHENTICATED PATH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Asked for in the Puffer Fish handoff, 2026-09-12. Only you can run this: it needs a real account, and creating accounts and typing passwords is outside what the sessions do.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>BEFORE YOU START</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Go to https://mothership-vtt.vercel.app  (NOT mothership.xerosumgames.com - the DNS record does not exist yet, that is a separate item). Comms verified 2026-09-12: the site returns 200, the sign-in form renders with Email, Password and Sign in, and "Create an account" switches it to Create account. Everything past that wall is what you are testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>THIS WRITES REAL DATA. You are creating a real account in the Mothership VTT Supabase project and a real character on it. Use an address you are happy to keep. Nothing here touches TheTapestry or TheTable accounts - the VTT has its own Supabase project by your own ruling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Have a .mothership.json file ready for the last step. If you do not have one, step 6 produces one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>What you do</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>What you should see if it is right</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="11" t="inlineStr"/>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Open https://mothership-vtt.vercel.app</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>The Mothership sign-in card: an Email box, a Password box, a Sign in button, "Create an account" below it, and a "The Table" link back to the hub.</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="11" t="inlineStr"/>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Click "Create an account"</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>The same card switches: the button now reads "Create account" and the link below reads "I already have an account". No page reload, no flicker to a different layout.</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="11" t="inlineStr"/>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Enter an email and password, click Create account</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>You end up signed in, or you are told to confirm your email. If it asks for confirmation, confirm it and come back - if the confirmation link errors, STOP and tell Comms: that is the redirect-URL allow-list, the same fault TheTable had.</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="11" t="inlineStr"/>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Once signed in, let the character sheet load</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>A character sheet, not an empty page and not a spinner that never resolves. Your class, stats and saves are on it.</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="11" t="inlineStr"/>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Roll something on the sheet</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>The rolled value appears and the sheet updates. Whatever you rolled reads as a number, not blank and not NaN.</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="C16" s="11" t="inlineStr"/>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Wait a moment, then reload the page without touching anything else</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>The sheet comes back exactly as you left it, including the roll from step 5. This is the autosave - if the roll is gone, autosave did not fire and that is the defect this test exists to catch.</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="C17" s="11" t="inlineStr"/>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Sign out</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>You are returned to the sign-in card from step 1. Your character is NOT visible while signed out.</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" s="11" t="inlineStr"/>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>Sign back in with the same account</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>The same character loads, with the same values. Not a fresh blank sheet, and not somebody else’s.</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="C19" s="11" t="inlineStr"/>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>Export or download the character as a .mothership.json file, if the sheet offers it</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="inlineStr">
+        <is>
+          <t>A file downloads. If there is no export control anywhere on the sheet, write that in Notes and skip to step 10 - Comms will file it.</t>
+        </is>
+      </c>
+      <c r="F19" s="11" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="11" t="inlineStr"/>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>Import a .mothership.json file</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>The imported character loads onto the sheet with its own values. Nothing is silently blank, and it does not overwrite a character you wanted to keep without telling you first.</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="8" t="inlineStr">
+        <is>
+          <t>IF ANYTHING FAILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Write what you actually saw in the row, and stop there rather than working around it. Tell Comms which step number failed - the step numbers are the whole point. A failure at step 3 is an auth-config problem, at step 6 an autosave problem, and at step 8 a persistence problem, and they go to different fixes.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C11:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Skipped"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
comms: fix the workbook formatting - merge prose across the table, set row heights
Prose was written into a 5-wide column B and rendered one character per line.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Table Smoke Testing.xlsx
+++ b/tasks/The Table Smoke Testing.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,8 +60,11 @@
       <b val="1"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +74,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
   </fills>
@@ -100,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,6 +142,32 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,63 +535,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B13"/>
+  <dimension ref="B1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="1"/>
+    <row r="2" ht="24" customHeight="1">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>THE TABLE - SMOKE TESTING</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="3"/>
+    <row r="4" ht="46.5" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>One living workbook. Your Pass/Fail marks are saved - reopen this file anytime and pick up where you left off. Every new test ask becomes a new worksheet in THIS file - never a new file, never a markdown test plan.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="3" t="inlineStr">
+    <row r="5"/>
+    <row r="6" ht="17" customHeight="1">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>HOW A TEST TAB READS</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="46.5" customHeight="1">
       <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Each tab is named for the ask and dated. Columns: Item | Status | Do this | What you saw | Notes. Steps are in the order you do them. Every step says what to do and what you should see if it is right. Anything you must set up first, or anything that changes saved data, is flagged at the top of the tab.</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" s="3" t="inlineStr">
+    <row r="8"/>
+    <row r="9" ht="17" customHeight="1">
+      <c r="B9" s="21" t="inlineStr">
         <is>
           <t>STATUS RIGHT NOW</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="46.5" customHeight="1">
       <c r="B10" s="5" t="inlineStr">
         <is>
           <t>One test tab is waiting on you: "Mothership VTT auth 2026-09-12" - the authenticated path on the Mothership VTT. It needs a real account, so only you can run it. Comms verified the site is up and the sign-in form renders before asking. Ten steps, each with what you should see.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="3" t="inlineStr">
+    <row r="11"/>
+    <row r="12" ht="17" customHeight="1">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>WHO MAINTAINS THIS</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="31" customHeight="1">
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Table | Comms owns this workbook and tasks/COMMS.md. Lanes route test asks and questions to Comms; Comms verifies a thing is actually reachable before asking you to look, then packages it here.</t>
@@ -560,6 +607,16 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="B13:E13"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B10:E10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -570,49 +627,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B10"/>
+  <dimension ref="B1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="2">
+    <row r="1"/>
+    <row r="2" ht="24" customHeight="1">
       <c r="B2" s="4" t="inlineStr">
         <is>
           <t>PROBE NOTES - for lanes, not for Xero</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="3"/>
+    <row r="4" ht="31" customHeight="1">
       <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Traps that have already produced a false test result. Read before writing an automated probe against a generator. Nothing here needs Xero to do anything.</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="5"/>
+    <row r="6" ht="17" customHeight="1">
       <c r="B6" s="6" t="inlineStr">
         <is>
           <t>1. Anything a probe injects into the page needs class="no-print"</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="46.5" customHeight="1">
       <c r="B7" s="5" t="inlineStr">
         <is>
           <t>A results div appended to document.body is not covered by these generators' print CSS, so it prints as a phantom second page and reads as a layout bug that is not there. This bit the Planet of the Apes sheet, then nearly caused a false report on Walking Dead. Added 2026-09-11 by Character Generators.</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="8"/>
+    <row r="9" ht="17" customHeight="1">
       <c r="B9" s="6" t="inlineStr">
         <is>
           <t>2. Print output IS reachable headless - print-to-PDF is not a substitute, it is the real thing</t>
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="62" customHeight="1">
       <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Print-to-PDF renders exactly what the print path produces; rasterise it and read it. Only the interactive print dialog and a real printer driver are out of reach. Do not file "needs a real print preview" as a blocker, and do not spend one of Xero's test slots on a paper check that a lane can do itself. Correction recorded 2026-09-11 by Character Generators, after the walkingdead print item was closed this way.</t>
@@ -620,6 +684,14 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B10:E10"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -630,271 +702,289 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F23"/>
+  <dimension ref="B1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="52" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="2">
-      <c r="B2" s="7" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>MOTHERSHIP VTT - THE AUTHENTICATED PATH</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="B3" s="5" t="inlineStr">
+    <row r="2" ht="31" customHeight="1">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Asked for in the Puffer Fish handoff, 2026-09-12. Only you can run this: it needs a real account, and creating accounts and typing passwords is outside what the sessions do.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="8" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="12" t="inlineStr">
         <is>
           <t>BEFORE YOU START</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="5" ht="17" customHeight="1">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Go to  https://mothership-vtt.vercel.app  -  NOT mothership.xerosumgames.com, whose DNS record does not exist yet (that is Q2, a separate item).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Go to https://mothership-vtt.vercel.app  (NOT mothership.xerosumgames.com - the DNS record does not exist yet, that is a separate item). Comms verified 2026-09-12: the site returns 200, the sign-in form renders with Email, Password and Sign in, and "Create an account" switches it to Create account. Everything past that wall is what you are testing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>THIS WRITES REAL DATA. You are creating a real account in the Mothership VTT Supabase project and a real character on it. Use an address you are happy to keep. Nothing here touches TheTapestry or TheTable accounts - the VTT has its own Supabase project by your own ruling.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Verified by Comms 2026-09-12: the site returns 200 and the sign-in card renders with Email, Password and Sign in, and "Create an account" switches it to Create account. Everything past that wall is what you are testing - the auth wall is where a session has to stop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="31" customHeight="1">
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>THIS WRITES REAL DATA. You are creating a real account in the Mothership VTT Supabase project, and a real character on it. Use an address you are happy to keep. Nothing here touches TheTapestry or TheTable accounts - the VTT has its own Supabase project, by your own ruling.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Have a .mothership.json file ready for the last step. If you do not have one, step 6 produces one.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="9" t="inlineStr">
+          <t>Have a .mothership.json file ready for the last step. If you do not have one, step 9 produces it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>Pass / Fail</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>What you do</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>What you should see if it is right</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="10" t="n">
+    <row r="11" ht="46.5" customHeight="1">
+      <c r="B11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="11" t="inlineStr"/>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr"/>
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>Open https://mothership-vtt.vercel.app</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="19" t="inlineStr">
         <is>
           <t>The Mothership sign-in card: an Email box, a Password box, a Sign in button, "Create an account" below it, and a "The Table" link back to the hub.</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="10" t="n">
+      <c r="F11" s="19" t="inlineStr"/>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="B12" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="inlineStr"/>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="C12" s="18" t="inlineStr"/>
+      <c r="D12" s="19" t="inlineStr">
         <is>
           <t>Click "Create an account"</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>The same card switches: the button now reads "Create account" and the link below reads "I already have an account". No page reload, no flicker to a different layout.</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="10" t="n">
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>The same card switches in place: the button now reads "Create account", the link below reads "I already have an account". No page reload, no jump to a different layout.</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr"/>
+    </row>
+    <row r="13" ht="62" customHeight="1">
+      <c r="B13" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="11" t="inlineStr"/>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="C13" s="18" t="inlineStr"/>
+      <c r="D13" s="19" t="inlineStr">
         <is>
           <t>Enter an email and password, click Create account</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>You end up signed in, or you are told to confirm your email. If it asks for confirmation, confirm it and come back - if the confirmation link errors, STOP and tell Comms: that is the redirect-URL allow-list, the same fault TheTable had.</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="10" t="n">
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Either you land signed in, or you are told to confirm your email. IF THE CONFIRMATION LINK ERRORS, STOP and tell Comms - that is the Supabase redirect-URL allow-list, the same fault TheTable had.</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr"/>
+    </row>
+    <row r="14" ht="46.5" customHeight="1">
+      <c r="B14" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="11" t="inlineStr"/>
-      <c r="D14" s="11" t="inlineStr">
+      <c r="C14" s="18" t="inlineStr"/>
+      <c r="D14" s="19" t="inlineStr">
         <is>
           <t>Once signed in, let the character sheet load</t>
         </is>
       </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>A character sheet, not an empty page and not a spinner that never resolves. Your class, stats and saves are on it.</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="10" t="n">
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>A character sheet - not an empty page, not a spinner that never resolves. Your class, stats and saves are on it.</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr"/>
+    </row>
+    <row r="15" ht="31" customHeight="1">
+      <c r="B15" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr"/>
+      <c r="D15" s="19" t="inlineStr">
         <is>
           <t>Roll something on the sheet</t>
         </is>
       </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>The rolled value appears and the sheet updates. Whatever you rolled reads as a number, not blank and not NaN.</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="10" t="n">
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>The rolled value appears and the sheet updates. It reads as a number, not blank and not NaN.</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr"/>
+    </row>
+    <row r="16" ht="62" customHeight="1">
+      <c r="B16" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="C16" s="11" t="inlineStr"/>
-      <c r="D16" s="11" t="inlineStr">
-        <is>
-          <t>Wait a moment, then reload the page without touching anything else</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>The sheet comes back exactly as you left it, including the roll from step 5. This is the autosave - if the roll is gone, autosave did not fire and that is the defect this test exists to catch.</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="10" t="n">
+      <c r="C16" s="18" t="inlineStr"/>
+      <c r="D16" s="19" t="inlineStr">
+        <is>
+          <t>Wait a moment, then reload the page. Do not touch anything else first.</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>The sheet returns exactly as you left it, INCLUDING the roll from step 5. This is the autosave. If the roll is gone, autosave did not fire - that is the defect this test exists to catch.</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr"/>
+    </row>
+    <row r="17" ht="31" customHeight="1">
+      <c r="B17" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="C17" s="11" t="inlineStr"/>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr"/>
+      <c r="D17" s="19" t="inlineStr">
         <is>
           <t>Sign out</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="19" t="inlineStr">
         <is>
           <t>You are returned to the sign-in card from step 1. Your character is NOT visible while signed out.</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="10" t="n">
+      <c r="F17" s="19" t="inlineStr"/>
+    </row>
+    <row r="18" ht="31" customHeight="1">
+      <c r="B18" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="C18" s="11" t="inlineStr"/>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="C18" s="18" t="inlineStr"/>
+      <c r="D18" s="19" t="inlineStr">
         <is>
           <t>Sign back in with the same account</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>The same character loads, with the same values. Not a fresh blank sheet, and not somebody else’s.</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="10" t="n">
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>The same character loads with the same values. Not a fresh blank sheet, and not somebody else’s.</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr"/>
+    </row>
+    <row r="19" ht="46.5" customHeight="1">
+      <c r="B19" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="11" t="inlineStr"/>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="C19" s="18" t="inlineStr"/>
+      <c r="D19" s="19" t="inlineStr">
         <is>
           <t>Export or download the character as a .mothership.json file, if the sheet offers it</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
-        <is>
-          <t>A file downloads. If there is no export control anywhere on the sheet, write that in Notes and skip to step 10 - Comms will file it.</t>
-        </is>
-      </c>
-      <c r="F19" s="11" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="10" t="n">
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>A file downloads. If there is no export control anywhere on the sheet, write that in Notes, skip to step 10 and Comms will file it as a gap.</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr"/>
+    </row>
+    <row r="20" ht="62" customHeight="1">
+      <c r="B20" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="C20" s="11" t="inlineStr"/>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="C20" s="18" t="inlineStr"/>
+      <c r="D20" s="19" t="inlineStr">
         <is>
           <t>Import a .mothership.json file</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>The imported character loads onto the sheet with its own values. Nothing is silently blank, and it does not overwrite a character you wanted to keep without telling you first.</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="8" t="inlineStr">
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>The imported character loads with its own values. Nothing silently blank, and it does not overwrite a character you wanted to keep without warning you first.</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr"/>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>IF ANYTHING FAILS</t>
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="46.5" customHeight="1">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Write what you actually saw in the row, and stop there rather than working around it. Tell Comms which step number failed - the step numbers are the whole point. A failure at step 3 is an auth-config problem, at step 6 an autosave problem, and at step 8 a persistence problem, and they go to different fixes.</t>
+          <t>Write what you actually saw in that row and stop there, rather than working around it. Tell Comms the step NUMBER - that is the whole point of them. A failure at step 3 is an auth-config problem, at step 6 an autosave problem, at step 8 a persistence problem, and they go to three different fixes.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B22:F22"/>
+  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C11:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pass,Fail,Skipped"</formula1>

</xml_diff>

<commit_message>
comms: add Incomplete to the smoke-test status values, fix the roll step
Xero's run marked step 5 Fail with "uncertain how to roll something" - a broken
step, not a defect. Reworded with a self-rescue clause and added a marking
legend. His Pass/Fail marks preserved.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Table Smoke Testing.xlsx
+++ b/tasks/The Table Smoke Testing.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,14 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mothership VTT auth 2026-09-12" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,26 +41,36 @@
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="18"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="16"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="12"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -73,17 +82,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDEDED"/>
+        <fgColor rgb="FFE8E8E8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8E8E8"/>
+        <fgColor rgb="FFFFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="00EAF3EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,82 +106,72 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </left>
       <right style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </right>
       <top style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D9D9D9"/>
+        <color rgb="FFD9D9D9"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -244,6 +243,52 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>6</col>
+      <colOff>19050</colOff>
+      <row>12</row>
+      <rowOff>9525</rowOff>
+    </from>
+    <to>
+      <col>26</col>
+      <colOff>39804</colOff>
+      <row>41</row>
+      <rowOff>38955</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Picture 1"/>
+        <cNvPicPr>
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </cNvPicPr>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="16306800" y="2381250"/>
+          <a:ext cx="12212754" cy="6125430"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <avLst/>
+        </a:prstGeom>
+        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -535,72 +580,65 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G13"/>
+  <dimension ref="B2:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
-    <col width="2" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
-    <col width="2" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" style="6" min="1" max="1"/>
+    <col width="100" customWidth="1" style="6" min="2" max="2"/>
+    <col width="2" customWidth="1" style="6" min="3" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="20" t="inlineStr">
+    <row r="2" ht="24" customHeight="1" s="6">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>THE TABLE - SMOKE TESTING</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="46.5" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
+    <row r="4" ht="46.5" customHeight="1" s="6">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>One living workbook. Your Pass/Fail marks are saved - reopen this file anytime and pick up where you left off. Every new test ask becomes a new worksheet in THIS file - never a new file, never a markdown test plan.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6" ht="17" customHeight="1">
-      <c r="B6" s="21" t="inlineStr">
+    <row r="6" ht="17.1" customHeight="1" s="6">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>HOW A TEST TAB READS</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46.5" customHeight="1">
-      <c r="B7" s="2" t="inlineStr">
+    <row r="7" ht="46.5" customHeight="1" s="6">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Each tab is named for the ask and dated. Columns: Item | Status | Do this | What you saw | Notes. Steps are in the order you do them. Every step says what to do and what you should see if it is right. Anything you must set up first, or anything that changes saved data, is flagged at the top of the tab.</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9" ht="17" customHeight="1">
-      <c r="B9" s="21" t="inlineStr">
+    <row r="9" ht="17.1" customHeight="1" s="6">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>STATUS RIGHT NOW</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="46.5" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+    <row r="10" ht="46.5" customHeight="1" s="6">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>One test tab is waiting on you: "Mothership VTT auth 2026-09-12" - the authenticated path on the Mothership VTT. It needs a real account, so only you can run it. Comms verified the site is up and the sign-in form renders before asking. Ten steps, each with what you should see.</t>
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12" ht="17" customHeight="1">
-      <c r="B12" s="21" t="inlineStr">
+    <row r="12" ht="17.1" customHeight="1" s="6">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>WHO MAINTAINS THIS</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="31" customHeight="1">
-      <c r="B13" s="2" t="inlineStr">
+    <row r="13" ht="30.95" customHeight="1" s="6">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Table | Comms owns this workbook and tasks/COMMS.md. Lanes route test asks and questions to Comms; Comms verifies a thing is actually reachable before asking you to look, then packages it here.</t>
         </is>
@@ -627,57 +665,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G10"/>
+  <dimension ref="B2:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
-    <col width="2" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
-    <col width="2" customWidth="1" min="5" max="5"/>
+    <col width="2" customWidth="1" style="6" min="1" max="1"/>
+    <col width="100" customWidth="1" style="6" min="2" max="2"/>
+    <col width="2" customWidth="1" style="6" min="3" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="24" customHeight="1">
-      <c r="B2" s="4" t="inlineStr">
+    <row r="2" ht="24" customHeight="1" s="6">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>PROBE NOTES - for lanes, not for Xero</t>
         </is>
       </c>
     </row>
-    <row r="3"/>
-    <row r="4" ht="31" customHeight="1">
-      <c r="B4" s="5" t="inlineStr">
+    <row r="4" ht="30.95" customHeight="1" s="6">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Traps that have already produced a false test result. Read before writing an automated probe against a generator. Nothing here needs Xero to do anything.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6" ht="17" customHeight="1">
-      <c r="B6" s="6" t="inlineStr">
+    <row r="6" ht="17.1" customHeight="1" s="6">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>1. Anything a probe injects into the page needs class="no-print"</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="46.5" customHeight="1">
-      <c r="B7" s="5" t="inlineStr">
+    <row r="7" ht="46.5" customHeight="1" s="6">
+      <c r="B7" s="9" t="inlineStr">
         <is>
           <t>A results div appended to document.body is not covered by these generators' print CSS, so it prints as a phantom second page and reads as a layout bug that is not there. This bit the Planet of the Apes sheet, then nearly caused a false report on Walking Dead. Added 2026-09-11 by Character Generators.</t>
         </is>
       </c>
     </row>
-    <row r="8"/>
-    <row r="9" ht="17" customHeight="1">
-      <c r="B9" s="6" t="inlineStr">
+    <row r="9" ht="17.1" customHeight="1" s="6">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>2. Print output IS reachable headless - print-to-PDF is not a substitute, it is the real thing</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="B10" s="5" t="inlineStr">
+    <row r="10" ht="62.1" customHeight="1" s="6">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Print-to-PDF renders exactly what the print path produces; rasterise it and read it. Only the interactive print dialog and a real printer driver are out of reach. Do not file "needs a real print preview" as a blocker, and do not spend one of Xero's test slots on a paper check that a lane can do itself. Correction recorded 2026-09-11 by Character Generators, after the walkingdead print item was closed this way.</t>
         </is>
@@ -702,294 +734,358 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F23"/>
+  <dimension ref="B1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="5" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="2" customWidth="1" style="6" min="1" max="1"/>
+    <col width="3" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="9.7109375" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="47.5703125" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="175.7109375" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="68" customWidth="1" style="6" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
-      <c r="B1" s="7" t="inlineStr">
+    <row r="1" ht="21.75" customHeight="1" s="6">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>MOTHERSHIP VTT - THE AUTHENTICATED PATH</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="31" customHeight="1">
-      <c r="B2" s="5" t="inlineStr">
+    <row r="2">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>Asked for in the Puffer Fish handoff, 2026-09-12. Only you can run this: it needs a real account, and creating accounts and typing passwords is outside what the sessions do.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
+    <row r="3"/>
+    <row r="4">
       <c r="B4" s="12" t="inlineStr">
         <is>
           <t>BEFORE YOU START</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="B5" s="5" t="inlineStr">
+    <row r="5">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Go to  https://mothership-vtt.vercel.app  -  NOT mothership.xerosumgames.com, whose DNS record does not exist yet (that is Q2, a separate item).</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="31" customHeight="1">
-      <c r="B6" s="5" t="inlineStr">
+    <row r="6">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Verified by Comms 2026-09-12: the site returns 200 and the sign-in card renders with Email, Password and Sign in, and "Create an account" switches it to Create account. Everything past that wall is what you are testing - the auth wall is where a session has to stop.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="31" customHeight="1">
-      <c r="B7" s="14" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>THIS WRITES REAL DATA. You are creating a real account in the Mothership VTT Supabase project, and a real character on it. Use an address you are happy to keep. Nothing here touches TheTapestry or TheTable accounts - the VTT has its own Supabase project, by your own ruling.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="B8" s="5" t="inlineStr">
+    <row r="8">
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>Have a .mothership.json file ready for the last step. If you do not have one, step 9 produces it.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="16" t="inlineStr">
+    <row r="9" ht="46.5" customHeight="1" s="6">
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>MARKING: Pass = it did what the row said. Fail = it did not, and you saw enough to say so. Skipped = you chose not to run it. Incomplete = you could not run it, because an earlier step blocked it or you could not find the control the step names. Incomplete is not a failure - it means nothing was proven either way, and it tells Comms to fix the step rather than chase a bug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Pass / Fail</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>What you do</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>What you should see if it is right</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="46.5" customHeight="1">
-      <c r="B11" s="17" t="n">
+    <row r="12">
+      <c r="B12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="18" t="inlineStr"/>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>Open https://mothership-vtt.vercel.app</t>
         </is>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>The Mothership sign-in card: an Email box, a Password box, a Sign in button, "Create an account" below it, and a "The Table" link back to the hub.</t>
         </is>
       </c>
-      <c r="F11" s="19" t="inlineStr"/>
-    </row>
-    <row r="12" ht="62" customHeight="1">
-      <c r="B12" s="17" t="n">
+      <c r="F12" s="4" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1" s="6">
+      <c r="B13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="18" t="inlineStr"/>
-      <c r="D12" s="19" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Click "Create an account"</t>
         </is>
       </c>
-      <c r="E12" s="19" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>The same card switches in place: the button now reads "Create account", the link below reads "I already have an account". No page reload, no jump to a different layout.</t>
         </is>
       </c>
-      <c r="F12" s="19" t="inlineStr"/>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="B13" s="17" t="n">
+      <c r="F13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="inlineStr"/>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Enter an email and password, click Create account</t>
         </is>
       </c>
-      <c r="E13" s="19" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>Either you land signed in, or you are told to confirm your email. IF THE CONFIRMATION LINK ERRORS, STOP and tell Comms - that is the Supabase redirect-URL allow-list, the same fault TheTable had.</t>
         </is>
       </c>
-      <c r="F13" s="19" t="inlineStr"/>
-    </row>
-    <row r="14" ht="46.5" customHeight="1">
-      <c r="B14" s="17" t="n">
+      <c r="F14" s="4" t="n"/>
+    </row>
+    <row r="15" ht="62" customHeight="1" s="6">
+      <c r="B15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="18" t="inlineStr"/>
-      <c r="D14" s="19" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Once signed in, let the character sheet load</t>
         </is>
       </c>
-      <c r="E14" s="19" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>A character sheet - not an empty page, not a spinner that never resolves. Your class, stats and saves are on it.</t>
         </is>
       </c>
-      <c r="F14" s="19" t="inlineStr"/>
-    </row>
-    <row r="15" ht="31" customHeight="1">
-      <c r="B15" s="17" t="n">
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>should be a dark/light button</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="6">
+      <c r="B16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="18" t="inlineStr"/>
-      <c r="D15" s="19" t="inlineStr">
-        <is>
-          <t>Roll something on the sheet</t>
-        </is>
-      </c>
-      <c r="E15" s="19" t="inlineStr">
-        <is>
-          <t>The rolled value appears and the sheet updates. It reads as a number, not blank and not NaN.</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="inlineStr"/>
-    </row>
-    <row r="16" ht="62" customHeight="1">
-      <c r="B16" s="17" t="n">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>Find anything on the sheet you can roll - a Stat, a Save, or a dice control - and roll it. If you cannot find ANY way to roll, mark this Incomplete and write that in Notes.</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>The rolled value appears and the sheet updates. It reads as a number, not blank and not NaN. If there is no roll control anywhere, that is the finding - the sheet is meant to have one.</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>uncertain how to "roll" something</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="C16" s="18" t="inlineStr"/>
-      <c r="D16" s="19" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>Wait a moment, then reload the page. Do not touch anything else first.</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>The sheet returns exactly as you left it, INCLUDING the roll from step 5. This is the autosave. If the roll is gone, autosave did not fire - that is the defect this test exists to catch.</t>
         </is>
       </c>
-      <c r="F16" s="19" t="inlineStr"/>
-    </row>
-    <row r="17" ht="31" customHeight="1">
-      <c r="B17" s="17" t="n">
+      <c r="F17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="C17" s="18" t="inlineStr"/>
-      <c r="D17" s="19" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>Sign out</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>You are returned to the sign-in card from step 1. Your character is NOT visible while signed out.</t>
         </is>
       </c>
-      <c r="F17" s="19" t="inlineStr"/>
-    </row>
-    <row r="18" ht="31" customHeight="1">
-      <c r="B18" s="17" t="n">
+      <c r="F18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="30" customHeight="1" s="6">
+      <c r="B19" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C18" s="18" t="inlineStr"/>
-      <c r="D18" s="19" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Sign back in with the same account</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>The same character loads with the same values. Not a fresh blank sheet, and not somebody else’s.</t>
         </is>
       </c>
-      <c r="F18" s="19" t="inlineStr"/>
-    </row>
-    <row r="19" ht="46.5" customHeight="1">
-      <c r="B19" s="17" t="n">
+      <c r="F19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C19" s="18" t="inlineStr"/>
-      <c r="D19" s="19" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>Export or download the character as a .mothership.json file, if the sheet offers it</t>
         </is>
       </c>
-      <c r="E19" s="19" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>A file downloads. If there is no export control anywhere on the sheet, write that in Notes, skip to step 10 and Comms will file it as a gap.</t>
         </is>
       </c>
-      <c r="F19" s="19" t="inlineStr"/>
-    </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="B20" s="17" t="n">
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>no export button visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="C20" s="18" t="inlineStr"/>
-      <c r="D20" s="19" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Skipped</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>Import a .mothership.json file</t>
         </is>
       </c>
-      <c r="E20" s="19" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>The imported character loads with its own values. Nothing silently blank, and it does not overwrite a character you wanted to keep without warning you first.</t>
         </is>
       </c>
-      <c r="F20" s="19" t="inlineStr"/>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="B22" s="12" t="inlineStr">
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22"/>
+    <row r="23">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>IF ANYTHING FAILS</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="46.5" customHeight="1">
-      <c r="B23" s="5" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Write what you actually saw in that row and stop there, rather than working around it. Tell Comms the step NUMBER - that is the whole point of them. A failure at step 3 is an auth-config problem, at step 6 an autosave problem, at step 8 a persistence problem, and they go to three different fixes.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B22:F22"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B9:F9"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C11:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pass,Fail,Skipped"</formula1>
+    <dataValidation sqref="C12:C21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Skipped,Incomplete"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
smoke: add the Mothership rerun tab after verifying the hub's push live
Signup redirect, light default and masthead shipped in bdba267; checked on
production before asking Xero to test.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Table Smoke Testing.xlsx
+++ b/tasks/The Table Smoke Testing.xlsx
@@ -9,6 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROBE NOTES" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mothership VTT auth 2026-09-12" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mothership rerun 2026-09-13" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +74,22 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -96,8 +111,18 @@
         <fgColor rgb="FFEAF3EA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3CD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -120,11 +145,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -171,6 +210,32 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -626,10 +691,10 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="46.5" customHeight="1" s="7">
+    <row r="10" ht="48" customHeight="1" s="7">
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>One test tab is waiting on you: "Mothership VTT auth 2026-09-12" - the authenticated path on the Mothership VTT. It needs a real account, so only you can run it. Comms verified the site is up and the sign-in form renders before asking. Ten steps, each with what you should see.</t>
+          <t>One test tab is waiting on you: "Mothership rerun 2026-09-13". Nine steps, about ten minutes. It checks the signup email fix, light mode, your logo, and the buttons that did not exist during yesterday's test. The older tab, "Mothership VTT auth 2026-09-12", is finished and kept as the record.</t>
         </is>
       </c>
     </row>
@@ -1098,4 +1163,296 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="7" min="1" max="1"/>
+    <col width="5" customWidth="1" style="7" min="2" max="2"/>
+    <col width="12" customWidth="1" style="7" min="3" max="3"/>
+    <col width="50" customWidth="1" style="7" min="4" max="4"/>
+    <col width="50" customWidth="1" style="7" min="5" max="5"/>
+    <col width="24" customWidth="1" style="7" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1" s="7">
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>MOTHERSHIP VTT - RERUN AFTER THE FIXES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="31" customHeight="1" s="7">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>The hub shipped the signup email fix, light mode as the default, and your logo in the title bar. This tab checks those, plus the parts of yesterday's test that could not be judged fairly because the buttons did not exist yet. About ten minutes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4" ht="18" customHeight="1" s="7">
+      <c r="B4" s="19" t="inlineStr">
+        <is>
+          <t>BEFORE YOU START</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1" s="7">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Go to https://mothership.xerosumgames.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1" s="7">
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Use a DIFFERENT email address from last time - that one already has an account. If you use Gmail, adding +2 before the @ works and still lands in your inbox, for example yourname+2@gmail.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="31" customHeight="1" s="7">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Checked by Comms 2026-09-13 before asking: the new version is live, the page opens in light mode, and the signup code now sends the confirmation link back to this site instead of localhost. The real email is the one thing only you can prove.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1" s="7">
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>THIS WRITES REAL DATA: a second real account and a real character in the Mothership VTT. Nothing here touches TheTable or TheTapestry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1" s="7">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Step 6 is a KNOWN problem the hub has not fixed yet: your last roll disappears when you reload. Mark what you see, but it is not a new failure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+    <row r="11" ht="20" customHeight="1" s="7">
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>Pass / Fail</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="inlineStr">
+        <is>
+          <t>What you do</t>
+        </is>
+      </c>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>What you should see if it is right</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46.5" customHeight="1" s="7">
+      <c r="B12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="25" t="inlineStr"/>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>Open https://mothership.xerosumgames.com</t>
+        </is>
+      </c>
+      <c r="E12" s="26" t="inlineStr">
+        <is>
+          <t>A LIGHT cream page with the Mothership sign-in card in the middle. Not the black page from last time.</t>
+        </is>
+      </c>
+      <c r="F12" s="26" t="inlineStr"/>
+    </row>
+    <row r="13" ht="31" customHeight="1" s="7">
+      <c r="B13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="25" t="inlineStr"/>
+      <c r="D13" s="26" t="inlineStr">
+        <is>
+          <t>Click "Create an account", enter your new email and a password, click Create account</t>
+        </is>
+      </c>
+      <c r="E13" s="26" t="inlineStr">
+        <is>
+          <t>A message telling you to check your email to confirm the account.</t>
+        </is>
+      </c>
+      <c r="F13" s="26" t="inlineStr"/>
+    </row>
+    <row r="14" ht="93" customHeight="1" s="7">
+      <c r="B14" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="25" t="inlineStr"/>
+      <c r="D14" s="26" t="inlineStr">
+        <is>
+          <t>Open the confirmation email and click the link in it</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>THE KEY STEP. The address bar shows mothership.xerosumgames.com - NOT localhost - and you are signed in, or can now sign in. If you see "This site can't be reached" or localhost again, mark Fail and paste a screenshot with the address bar cropped off.</t>
+        </is>
+      </c>
+      <c r="F14" s="26" t="inlineStr"/>
+    </row>
+    <row r="15" ht="31" customHeight="1" s="7">
+      <c r="B15" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="25" t="inlineStr"/>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>Once signed in, look at the bar across the top of the app</t>
+        </is>
+      </c>
+      <c r="E15" s="26" t="inlineStr">
+        <is>
+          <t>The Mothership logo sits in the title bar. In light mode it is the dark version of the logo.</t>
+        </is>
+      </c>
+      <c r="F15" s="26" t="inlineStr"/>
+    </row>
+    <row r="16" ht="62" customHeight="1" s="7">
+      <c r="B16" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" s="25" t="inlineStr"/>
+      <c r="D16" s="26" t="inlineStr">
+        <is>
+          <t>Roll something on the sheet - a Stat, a Save, or a dice control</t>
+        </is>
+      </c>
+      <c r="E16" s="26" t="inlineStr">
+        <is>
+          <t>The result is easy to see, and it also appears in a Game log in the left sidebar. If you cannot find where the result shows, mark Incomplete and say so.</t>
+        </is>
+      </c>
+      <c r="F16" s="26" t="inlineStr"/>
+    </row>
+    <row r="17" ht="62" customHeight="1" s="7">
+      <c r="B17" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="C17" s="25" t="inlineStr"/>
+      <c r="D17" s="26" t="inlineStr">
+        <is>
+          <t>Reload the page</t>
+        </is>
+      </c>
+      <c r="E17" s="26" t="inlineStr">
+        <is>
+          <t>Your character comes back as it was. The last roll will probably be GONE from the log - that is the known problem from the warning above, so note it rather than marking Fail for it.</t>
+        </is>
+      </c>
+      <c r="F17" s="26" t="inlineStr"/>
+    </row>
+    <row r="18" ht="46.5" customHeight="1" s="7">
+      <c r="B18" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="C18" s="25" t="inlineStr"/>
+      <c r="D18" s="26" t="inlineStr">
+        <is>
+          <t>Look in the left sidebar for an Export button, and click it</t>
+        </is>
+      </c>
+      <c r="E18" s="26" t="inlineStr">
+        <is>
+          <t>A file ending .mothership.json downloads. If you cannot find an Export button anywhere, mark Incomplete and say where you looked.</t>
+        </is>
+      </c>
+      <c r="F18" s="26" t="inlineStr"/>
+    </row>
+    <row r="19" ht="31" customHeight="1" s="7">
+      <c r="B19" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="C19" s="25" t="inlineStr"/>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>In the same sidebar, look for New character and Random character. Click Random character</t>
+        </is>
+      </c>
+      <c r="E19" s="26" t="inlineStr">
+        <is>
+          <t>A different, fully rolled character appears. If you cannot find either button, mark Incomplete.</t>
+        </is>
+      </c>
+      <c r="F19" s="26" t="inlineStr"/>
+    </row>
+    <row r="20" ht="31" customHeight="1" s="7">
+      <c r="B20" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" s="25" t="inlineStr"/>
+      <c r="D20" s="26" t="inlineStr">
+        <is>
+          <t>Click Import and choose the file you exported in step 7</t>
+        </is>
+      </c>
+      <c r="E20" s="26" t="inlineStr">
+        <is>
+          <t>The exported character loads back in with the same name and values.</t>
+        </is>
+      </c>
+      <c r="F20" s="26" t="inlineStr"/>
+    </row>
+    <row r="21"/>
+    <row r="22" ht="18" customHeight="1" s="7">
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>IF ANYTHING FAILS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="31" customHeight="1" s="7">
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Tell Comms the step NUMBER. Step 3 is the signup email and matters most - a failure there means new players still cannot join. Steps 7 and 8 marked Incomplete mean the buttons are hard to find, which is a layout fix rather than a bug.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B9:F9"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C12:C20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pass,Fail,Skipped,Incomplete"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>